<commit_message>
Test.xlsx - Commented GitLatch Commit @ 2025-8-21-9-31-50-986
</commit_message>
<xml_diff>
--- a/pppppppp.xlsx
+++ b/pppppppp.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26021"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10720"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{01E3BBA4-F604-4985-B5CA-7BDFD924A46C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7C8A217A-53E4-054E-B538-0F6ED71A35C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="500" windowWidth="28000" windowHeight="14880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,9 +27,17 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+  <si>
+    <t>nnnn</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -78,9 +86,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -118,7 +126,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -224,7 +232,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -366,7 +374,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -401,9 +409,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
+  <dimension ref="N6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="6" spans="14:14" x14ac:dyDescent="0.2">
+      <c r="N6" t="s">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>